<commit_message>
docs(entrega-2): state the assumptions behind the cone
Velocity, team size, sample vacancies, no LinkedIn API, local deployment, and why Operate and Technical Items are zero.
</commit_message>
<xml_diff>
--- a/docs/deliverables/delivery-2/document/Entrega2_Template_HistoriasUsuario.xlsx
+++ b/docs/deliverables/delivery-2/document/Entrega2_Template_HistoriasUsuario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pablo/Library/Containers/com.microsoft.Excel/Data/tmp/ml/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42DD1CE2-21C4-7745-B942-0C911EDD63D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6A1E17F-A0CB-2B43-931D-C5A5FF1E8EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4880" yWindow="600" windowWidth="34500" windowHeight="22820" tabRatio="677" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -193,7 +193,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="164">
   <si>
     <t>Features backlog</t>
   </si>
@@ -692,6 +692,30 @@
   </si>
   <si>
     <t>#36 Logging without sensitive data</t>
+  </si>
+  <si>
+    <t>La velocidad promedio es de 50 puntos por sprint, la que logró el equipo en el Sprint 1.</t>
+  </si>
+  <si>
+    <t>El equipo son dos personas, con la misma disponibilidad en todos los sprints.</t>
+  </si>
+  <si>
+    <t>Los puntos de las historias de la fase Later no cambian al refinarlas.</t>
+  </si>
+  <si>
+    <t>Las vacantes vienen de un conjunto de prueba de 20, no de datos reales de Magneto.</t>
+  </si>
+  <si>
+    <t>No se cuenta con una API de LinkedIn que entregue la experiencia, la educación y las habilidades del perfil.</t>
+  </si>
+  <si>
+    <t>El despliegue local es suficiente para las entregas, como lo permite el reto.</t>
+  </si>
+  <si>
+    <t>Las historias no funcionales (#32 a #36) no se estiman en puntos, así que no entran en el cono.</t>
+  </si>
+  <si>
+    <t>No hay sprints de operación ni de puesta en producción, y el ambiente de desarrollo (Docker y el monorepo) existe desde el Sprint 1. Por eso Operate y Technical Items valen 0.</t>
   </si>
 </sst>
 </file>
@@ -2188,6 +2212,15 @@
     <xf numFmtId="2" fontId="18" fillId="44" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="43" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="43" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="43" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="47" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2227,15 +2260,6 @@
     <xf numFmtId="0" fontId="30" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="43" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="43" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="43" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2296,6 +2320,38 @@
   <dxfs count="38">
     <dxf>
       <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2328,6 +2384,30 @@
         <bottom style="medium">
           <color theme="0"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.34998626667073579"/>
+        </patternFill>
+      </fill>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
       </border>
     </dxf>
     <dxf>
@@ -2370,6 +2450,30 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.34998626667073579"/>
+        </patternFill>
+      </fill>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2402,6 +2506,41 @@
         </top>
         <bottom style="medium">
           <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFCA3B41"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
         </bottom>
       </border>
     </dxf>
@@ -2444,6 +2583,41 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF7BE66"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2476,6 +2650,41 @@
         </top>
         <bottom style="medium">
           <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF487B48"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
         </bottom>
       </border>
     </dxf>
@@ -2514,6 +2723,24 @@
         <bottom style="medium">
           <color theme="0"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border outline="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
       </border>
     </dxf>
     <dxf>
@@ -2557,42 +2784,16 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
         <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="0"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </right>
-        <top style="medium">
-          <color theme="0"/>
-        </top>
-        <bottom style="medium">
-          <color theme="0"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -2635,6 +2836,19 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2671,6 +2885,71 @@
           <color theme="0"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </right>
+        <top style="medium">
+          <color theme="0"/>
+        </top>
+        <bottom style="medium">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -2713,6 +2992,19 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2749,6 +3041,19 @@
           <color theme="0"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -2791,6 +3096,19 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2827,300 +3145,6 @@
           <color theme="0"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0.0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFCA3B41"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0.0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF7BE66"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0.0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF487B48"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border outline="0">
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -19448,28 +19472,28 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A2:N24" totalsRowCount="1" headerRowDxfId="37" dataDxfId="36" totalsRowDxfId="35" totalsRowBorderDxfId="34">
   <autoFilter ref="A2:N23" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" totalsRowLabel="Total" dataDxfId="33" totalsRowDxfId="13"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Capability" dataDxfId="32" totalsRowDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Backlog Item _x000a_(Feature or Story)" dataDxfId="31" totalsRowDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Comments" dataDxfId="30" totalsRowDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase" dataDxfId="29" totalsRowDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Tshirt Sizing" dataDxfId="28" totalsRowDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Story Points" dataDxfId="27" totalsRowDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Business Uncertainty" dataDxfId="26" totalsRowDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Technical Complexity" dataDxfId="25" totalsRowDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="BEST CASE" totalsRowFunction="sum" dataDxfId="24" totalsRowDxfId="4">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" totalsRowLabel="Total" dataDxfId="33" totalsRowDxfId="32"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Capability" dataDxfId="31" totalsRowDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Backlog Item _x000a_(Feature or Story)" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Comments" dataDxfId="27" totalsRowDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase" dataDxfId="25" totalsRowDxfId="24"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Tshirt Sizing" dataDxfId="23" totalsRowDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Story Points" dataDxfId="21" totalsRowDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Business Uncertainty" dataDxfId="19" totalsRowDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Technical Complexity" dataDxfId="17" totalsRowDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="BEST CASE" totalsRowFunction="sum" dataDxfId="15" totalsRowDxfId="14">
       <calculatedColumnFormula>IFERROR((K3-K3*M3),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="MOST LIKELY" totalsRowFunction="sum" dataDxfId="23" totalsRowDxfId="3">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="MOST LIKELY" totalsRowFunction="sum" dataDxfId="13" totalsRowDxfId="12">
       <calculatedColumnFormula>IFERROR((IF(ISBLANK(G3),VLOOKUP(F3,lst_TShirt_2_SP_Avg,2,FALSE),G3)),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="WORST CASE" totalsRowFunction="sum" dataDxfId="22" totalsRowDxfId="2">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="WORST CASE" totalsRowFunction="sum" dataDxfId="11" totalsRowDxfId="10">
       <calculatedColumnFormula>K3+K3*M3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="CONE of Uncertainty" dataDxfId="21" totalsRowDxfId="1">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="CONE of Uncertainty" dataDxfId="9" totalsRowDxfId="8">
       <calculatedColumnFormula>IF(H3="Low",VLOOKUP(N3,lst_tshirt_bu,2,FALSE),IF(H3="Medium",VLOOKUP(N3,lst_tshirt_bu,3,FALSE),IF(H3="High",VLOOKUP(N3,lst_tshirt_bu,4,FALSE),0))) + IF(I3="Low",VLOOKUP(N3,lst_tshirt_tc,2,FALSE),IF(I3="Medium",VLOOKUP(N3,lst_tshirt_tc,3,FALSE),IF(I3="High",VLOOKUP(N3,lst_tshirt_tc,4,FALSE),0)))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Tshirt Size for Cone Calc" dataDxfId="20" totalsRowDxfId="0">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Tshirt Size for Cone Calc" dataDxfId="7" totalsRowDxfId="6">
       <calculatedColumnFormula>IF(ISBLANK(G3),F3,VLOOKUP(G3,lst_SP_to_TShirt,2,FALSE))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -19827,22 +19851,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:87" ht="18" customHeight="1" thickBot="1">
-      <c r="A1" s="134" t="s">
+      <c r="A1" s="137" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="135"/>
-      <c r="C1" s="135"/>
-      <c r="D1" s="135"/>
-      <c r="E1" s="135"/>
-      <c r="F1" s="135"/>
-      <c r="G1" s="135"/>
-      <c r="H1" s="135"/>
-      <c r="I1" s="135"/>
-      <c r="J1" s="135"/>
-      <c r="K1" s="135"/>
-      <c r="L1" s="135"/>
-      <c r="M1" s="135"/>
-      <c r="N1" s="136"/>
+      <c r="B1" s="138"/>
+      <c r="C1" s="138"/>
+      <c r="D1" s="138"/>
+      <c r="E1" s="138"/>
+      <c r="F1" s="138"/>
+      <c r="G1" s="138"/>
+      <c r="H1" s="138"/>
+      <c r="I1" s="138"/>
+      <c r="J1" s="138"/>
+      <c r="K1" s="138"/>
+      <c r="L1" s="138"/>
+      <c r="M1" s="138"/>
+      <c r="N1" s="139"/>
     </row>
     <row r="2" spans="1:87" s="14" customFormat="1" ht="51">
       <c r="A2" s="23" t="s">
@@ -24999,23 +25023,23 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="A3:D23">
-    <cfRule type="expression" dxfId="19" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>COUNTBLANK($F3:$G3)=2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A25:M26 H2:I24 N26 O28:Q419 I27:N417">
-    <cfRule type="cellIs" dxfId="18" priority="2" operator="equal">
+  <conditionalFormatting sqref="H2:I24 A25:M26 N26 I27:N417 O28:Q419">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
       <formula>"High"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"Medium"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:L2 J24:L24 H27:I1048576">
-    <cfRule type="cellIs" dxfId="16" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="6" operator="equal">
       <formula>"High"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="7" operator="equal">
       <formula>"Medium"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25034,7 +25058,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N3:N23">
-    <cfRule type="expression" dxfId="14" priority="4">
+    <cfRule type="expression" dxfId="0" priority="4">
       <formula>N3&lt;&gt;F3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25117,28 +25141,28 @@
       <c r="C3" s="105"/>
     </row>
     <row r="4" spans="2:19" ht="16">
-      <c r="B4" s="137" t="s">
+      <c r="B4" s="140" t="s">
         <v>125</v>
       </c>
-      <c r="C4" s="138"/>
-      <c r="D4" s="138"/>
-      <c r="E4" s="138"/>
-      <c r="F4" s="138"/>
-      <c r="G4" s="139"/>
-      <c r="I4" s="137" t="s">
+      <c r="C4" s="141"/>
+      <c r="D4" s="141"/>
+      <c r="E4" s="141"/>
+      <c r="F4" s="141"/>
+      <c r="G4" s="142"/>
+      <c r="I4" s="140" t="s">
         <v>28</v>
       </c>
-      <c r="J4" s="138"/>
-      <c r="K4" s="138"/>
-      <c r="L4" s="138"/>
-      <c r="M4" s="138"/>
-      <c r="O4" s="137" t="s">
+      <c r="J4" s="141"/>
+      <c r="K4" s="141"/>
+      <c r="L4" s="141"/>
+      <c r="M4" s="141"/>
+      <c r="O4" s="140" t="s">
         <v>29</v>
       </c>
-      <c r="P4" s="138"/>
-      <c r="Q4" s="138"/>
-      <c r="R4" s="138"/>
-      <c r="S4" s="138"/>
+      <c r="P4" s="141"/>
+      <c r="Q4" s="141"/>
+      <c r="R4" s="141"/>
+      <c r="S4" s="141"/>
     </row>
     <row r="5" spans="2:19" ht="51">
       <c r="B5" s="26" t="s">
@@ -25591,7 +25615,7 @@
       </c>
     </row>
     <row r="3" spans="2:25" ht="0.75" customHeight="1">
-      <c r="C3" s="141" t="s">
+      <c r="C3" s="144" t="s">
         <v>40</v>
       </c>
       <c r="D3" s="117">
@@ -25608,7 +25632,7 @@
       <c r="U3" s="4"/>
     </row>
     <row r="4" spans="2:25" ht="16.25" customHeight="1">
-      <c r="C4" s="141"/>
+      <c r="C4" s="144"/>
       <c r="D4" s="117">
         <f>ROUNDUP(Table1[[#Totals],[BEST CASE]]/avgVelocity,0) + D14 +D15</f>
         <v>1</v>
@@ -25623,7 +25647,7 @@
       </c>
     </row>
     <row r="5" spans="2:25" ht="0.75" customHeight="1">
-      <c r="C5" s="142" t="s">
+      <c r="C5" s="145" t="s">
         <v>41</v>
       </c>
       <c r="D5" s="118">
@@ -25637,7 +25661,7 @@
       </c>
     </row>
     <row r="6" spans="2:25" ht="13.5" customHeight="1">
-      <c r="C6" s="142"/>
+      <c r="C6" s="145"/>
       <c r="D6" s="118">
         <f>ROUNDUP(Table1[[#Totals],[MOST LIKELY]]/avgVelocity,0) + D14 +D15</f>
         <v>2</v>
@@ -25652,7 +25676,7 @@
       </c>
     </row>
     <row r="7" spans="2:25" ht="15" hidden="1" customHeight="1">
-      <c r="C7" s="143" t="s">
+      <c r="C7" s="146" t="s">
         <v>42</v>
       </c>
       <c r="D7" s="119">
@@ -25666,7 +25690,7 @@
       </c>
     </row>
     <row r="8" spans="2:25">
-      <c r="C8" s="143"/>
+      <c r="C8" s="146"/>
       <c r="D8" s="119">
         <f>ROUNDUP(Table1[[#Totals],[WORST CASE]]/avgVelocity,0)  + D14 +D15</f>
         <v>2</v>
@@ -25681,7 +25705,7 @@
       </c>
     </row>
     <row r="9" spans="2:25" ht="0.75" customHeight="1">
-      <c r="C9" s="144" t="s">
+      <c r="C9" s="147" t="s">
         <v>43</v>
       </c>
       <c r="D9" s="120">
@@ -25696,7 +25720,7 @@
       </c>
     </row>
     <row r="10" spans="2:25" ht="16" thickBot="1">
-      <c r="C10" s="145"/>
+      <c r="C10" s="148"/>
       <c r="D10" s="133">
         <f>ROUNDUP(Table1[[#Totals],[MOST LIKELY]]/avgVelocity + 'Cone of Uncertainty'!D21,0)</f>
         <v>4</v>
@@ -25753,10 +25777,10 @@
       <c r="B16" s="55"/>
     </row>
     <row r="18" spans="3:4">
-      <c r="C18" s="140" t="s">
+      <c r="C18" s="143" t="s">
         <v>122</v>
       </c>
-      <c r="D18" s="140"/>
+      <c r="D18" s="143"/>
     </row>
     <row r="19" spans="3:4">
       <c r="C19" s="3" t="s">
@@ -26050,49 +26074,65 @@
       <c r="B3" s="3">
         <v>1</v>
       </c>
-      <c r="C3" s="3"/>
+      <c r="C3" s="3" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="4" spans="2:3">
       <c r="B4" s="3">
         <v>2</v>
       </c>
-      <c r="C4" s="3"/>
+      <c r="C4" s="3" t="s">
+        <v>157</v>
+      </c>
     </row>
     <row r="5" spans="2:3">
       <c r="B5" s="3">
         <v>3</v>
       </c>
-      <c r="C5" s="3"/>
+      <c r="C5" s="3" t="s">
+        <v>158</v>
+      </c>
     </row>
     <row r="6" spans="2:3">
       <c r="B6" s="3">
         <v>4</v>
       </c>
-      <c r="C6" s="3"/>
+      <c r="C6" s="3" t="s">
+        <v>159</v>
+      </c>
     </row>
     <row r="7" spans="2:3">
       <c r="B7" s="3">
         <v>5</v>
       </c>
-      <c r="C7" s="3"/>
+      <c r="C7" s="3" t="s">
+        <v>160</v>
+      </c>
     </row>
     <row r="8" spans="2:3">
       <c r="B8" s="3">
         <v>6</v>
       </c>
-      <c r="C8" s="3"/>
+      <c r="C8" s="3" t="s">
+        <v>161</v>
+      </c>
     </row>
     <row r="9" spans="2:3">
       <c r="B9" s="3">
         <v>7</v>
       </c>
-      <c r="C9" s="3"/>
+      <c r="C9" s="3" t="s">
+        <v>162</v>
+      </c>
     </row>
     <row r="10" spans="2:3">
       <c r="B10" s="3">
         <v>8</v>
       </c>
-      <c r="C10" s="3"/>
+      <c r="C10" s="3" t="s">
+        <v>163</v>
+      </c>
     </row>
     <row r="11" spans="2:3">
       <c r="B11" s="3">
@@ -26133,50 +26173,50 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20" ht="19.25" customHeight="1">
-      <c r="A1" s="146" t="s">
+      <c r="A1" s="149" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="146"/>
-      <c r="C1" s="146"/>
-      <c r="D1" s="146"/>
-      <c r="E1" s="146"/>
-      <c r="F1" s="146"/>
-      <c r="G1" s="146"/>
-      <c r="H1" s="146"/>
-      <c r="I1" s="146"/>
-      <c r="J1" s="146"/>
-      <c r="K1" s="146"/>
-      <c r="L1" s="146"/>
-      <c r="M1" s="146"/>
-      <c r="N1" s="146"/>
-      <c r="O1" s="146"/>
-      <c r="P1" s="146"/>
-      <c r="Q1" s="146"/>
-      <c r="R1" s="146"/>
-      <c r="S1" s="146"/>
-      <c r="T1" s="146"/>
+      <c r="B1" s="149"/>
+      <c r="C1" s="149"/>
+      <c r="D1" s="149"/>
+      <c r="E1" s="149"/>
+      <c r="F1" s="149"/>
+      <c r="G1" s="149"/>
+      <c r="H1" s="149"/>
+      <c r="I1" s="149"/>
+      <c r="J1" s="149"/>
+      <c r="K1" s="149"/>
+      <c r="L1" s="149"/>
+      <c r="M1" s="149"/>
+      <c r="N1" s="149"/>
+      <c r="O1" s="149"/>
+      <c r="P1" s="149"/>
+      <c r="Q1" s="149"/>
+      <c r="R1" s="149"/>
+      <c r="S1" s="149"/>
+      <c r="T1" s="149"/>
     </row>
     <row r="2" spans="1:20" ht="29" customHeight="1">
-      <c r="A2" s="146"/>
-      <c r="B2" s="146"/>
-      <c r="C2" s="146"/>
-      <c r="D2" s="146"/>
-      <c r="E2" s="146"/>
-      <c r="F2" s="146"/>
-      <c r="G2" s="146"/>
-      <c r="H2" s="146"/>
-      <c r="I2" s="146"/>
-      <c r="J2" s="146"/>
-      <c r="K2" s="146"/>
-      <c r="L2" s="146"/>
-      <c r="M2" s="146"/>
-      <c r="N2" s="146"/>
-      <c r="O2" s="146"/>
-      <c r="P2" s="146"/>
-      <c r="Q2" s="146"/>
-      <c r="R2" s="146"/>
-      <c r="S2" s="146"/>
-      <c r="T2" s="146"/>
+      <c r="A2" s="149"/>
+      <c r="B2" s="149"/>
+      <c r="C2" s="149"/>
+      <c r="D2" s="149"/>
+      <c r="E2" s="149"/>
+      <c r="F2" s="149"/>
+      <c r="G2" s="149"/>
+      <c r="H2" s="149"/>
+      <c r="I2" s="149"/>
+      <c r="J2" s="149"/>
+      <c r="K2" s="149"/>
+      <c r="L2" s="149"/>
+      <c r="M2" s="149"/>
+      <c r="N2" s="149"/>
+      <c r="O2" s="149"/>
+      <c r="P2" s="149"/>
+      <c r="Q2" s="149"/>
+      <c r="R2" s="149"/>
+      <c r="S2" s="149"/>
+      <c r="T2" s="149"/>
     </row>
     <row r="4" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="A4" s="56" t="s">
@@ -26424,11 +26464,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4">
-      <c r="B2" s="147" t="s">
+      <c r="B2" s="134" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="148"/>
-      <c r="D2" s="149"/>
+      <c r="C2" s="135"/>
+      <c r="D2" s="136"/>
     </row>
     <row r="3" spans="2:4" ht="14.25" customHeight="1">
       <c r="B3" s="116" t="s">
@@ -27147,21 +27187,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006DEE37CDC9AEA44CBD8F091652A6C5E4" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9de09e14d18b2e0769f00e11c33b035a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7bb3299b-b075-41c7-bb54-99fc85b15d4f" xmlns:ns3="08caf6cd-a550-4dce-b6c8-fe9b0e6bc4e3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="81a6a9a579b993e4978c34f4e71e25a5" ns2:_="" ns3:_="">
     <xsd:import namespace="7bb3299b-b075-41c7-bb54-99fc85b15d4f"/>
@@ -27372,24 +27397,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1010AAFC-6E8A-4F4B-91D1-B1DB8DD7131E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF49F70C-261C-4E13-A8B5-F2B201AA0A03}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D916E78-7E6F-4E04-B4AA-CEC365547DDB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -27406,4 +27429,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF49F70C-261C-4E13-A8B5-F2B201AA0A03}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1010AAFC-6E8A-4F4B-91D1-B1DB8DD7131E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
docs(entrega-2): replace the template's definition of done with the team's
Acceptance criteria, issue and branch, domain rules tested in core, review requested on the PR, the five checks green, and the board updated.
</commit_message>
<xml_diff>
--- a/docs/deliverables/delivery-2/document/Entrega2_Template_HistoriasUsuario.xlsx
+++ b/docs/deliverables/delivery-2/document/Entrega2_Template_HistoriasUsuario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pablo/Library/Containers/com.microsoft.Excel/Data/tmp/ml/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6A1E17F-A0CB-2B43-931D-C5A5FF1E8EDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D64F0FD-42B8-6143-A42D-7126D1496034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4880" yWindow="600" windowWidth="34500" windowHeight="22820" tabRatio="677" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -193,7 +193,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="133">
   <si>
     <t>Features backlog</t>
   </si>
@@ -360,163 +360,6 @@
   </si>
   <si>
     <t>Assumptions</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">This template uses an average velocity (Story Points) to calculate the cone of uncertainty (duration interval). For that to be valid you'll need the estimation team to allign on what "done" means and what activities are included. The below is an </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="16"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>example</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> as a starting points and should be tailored case-by-case</t>
-    </r>
-  </si>
-  <si>
-    <t>Development</t>
-  </si>
-  <si>
-    <t>Technical Implementation Plan confirmed with architects/TL [if needed].</t>
-  </si>
-  <si>
-    <t>Code written and tested locally.</t>
-  </si>
-  <si>
-    <t>Unit Tests developed for Back-end ( 80% code coverage) and Front-end ( 60% code coverage).</t>
-  </si>
-  <si>
-    <t>Code reviewed and approved by at least one mandatory approval.</t>
-  </si>
-  <si>
-    <t>Documentation of model/controllers/sequence diagrams [if needed].</t>
-  </si>
-  <si>
-    <t>IDs for FE elements ( where needed). - checked on code review &amp; testing.</t>
-  </si>
-  <si>
-    <t>Configuration check - (if needed ) added in release notes.</t>
-  </si>
-  <si>
-    <t>Release notes updated.</t>
-  </si>
-  <si>
-    <t>Sonar execution on review - no critical issues accepted.</t>
-  </si>
-  <si>
-    <t>English labels available in CMS ( if needed).</t>
-  </si>
-  <si>
-    <t>All defects reported by testing fixed.</t>
-  </si>
-  <si>
-    <t>Deployment/Demo</t>
-  </si>
-  <si>
-    <t>Changes deployed successfully to Openshift Director env (no build error + sonar passed successfully )  &gt;= 5 SP (2 days before sprint ends), only bug fixing will be allowed.</t>
-  </si>
-  <si>
-    <t>Deployment freeze also 3 hours before demo.</t>
-  </si>
-  <si>
-    <t>Testing</t>
-  </si>
-  <si>
-    <t>Test cases written in Zephyr.</t>
-  </si>
-  <si>
-    <t>Application tested against the mock layer, including error cases and edge.</t>
-  </si>
-  <si>
-    <t>Manual functional test 100% test coverage on test environment.</t>
-  </si>
-  <si>
-    <t>Manual test (basic and advanced) cases executed and passing.</t>
-  </si>
-  <si>
-    <t>Exploratory testing executed.</t>
-  </si>
-  <si>
-    <t>Testing passed 100% on Test Environment.</t>
-  </si>
-  <si>
-    <t>All issues reported as bugs and linked to the stories.</t>
-  </si>
-  <si>
-    <t>Acceptance criteria fulfilled.</t>
-  </si>
-  <si>
-    <t>Test data is documented.</t>
-  </si>
-  <si>
-    <t>NFR fulfilled.</t>
-  </si>
-  <si>
-    <t>Quality Acceptance.</t>
-  </si>
-  <si>
-    <t>No issues with severity worse than Major.</t>
-  </si>
-  <si>
-    <t>Feature documented in TBD owner.</t>
-  </si>
-  <si>
-    <t>User story is updated with latest information/requirements.</t>
-  </si>
-  <si>
-    <t>Automated testing</t>
-  </si>
-  <si>
-    <t>Automated tests written.</t>
-  </si>
-  <si>
-    <t>Automated tests committed to Git.</t>
-  </si>
-  <si>
-    <t>Automated tests executed and validated.</t>
-  </si>
-  <si>
-    <t>Other considerations</t>
-  </si>
-  <si>
-    <t>(TBD story by story</t>
-  </si>
-  <si>
-    <t>OR add a separate story)</t>
-  </si>
-  <si>
-    <t>*all to be covered with Acceptance criteria.</t>
-  </si>
-  <si>
-    <t>Performance.</t>
-  </si>
-  <si>
-    <t>Security.</t>
-  </si>
-  <si>
-    <t>Error handling.</t>
-  </si>
-  <si>
-    <t>Localization.</t>
-  </si>
-  <si>
-    <t>In-house usability testing.</t>
   </si>
   <si>
     <t>Delivery Team(s) Shape</t>
@@ -716,6 +559,45 @@
   </si>
   <si>
     <t>No hay sprints de operación ni de puesta en producción, y el ambiente de desarrollo (Docker y el monorepo) existe desde el Sprint 1. Por eso Operate y Technical Items valen 0.</t>
+  </si>
+  <si>
+    <t>Una historia cuenta como terminada, y suma a la velocidad del cono, solo cuando cumple todo lo de esta hoja.</t>
+  </si>
+  <si>
+    <t>Desarrollo</t>
+  </si>
+  <si>
+    <t>Los criterios de aceptación de la historia se cumplen todos.</t>
+  </si>
+  <si>
+    <t>La historia tiene su issue y su propia rama, creada desde main.</t>
+  </si>
+  <si>
+    <t>Las reglas del dominio viven en packages/core y tienen pruebas; el SQL vive solo en packages/db.</t>
+  </si>
+  <si>
+    <t>Revisión</t>
+  </si>
+  <si>
+    <t>El PR enlaza su issue con Closes #N y pide la revisión del otro integrante.</t>
+  </si>
+  <si>
+    <t>Se integra con squash merge y la rama se borra.</t>
+  </si>
+  <si>
+    <t>Pruebas</t>
+  </si>
+  <si>
+    <t>Pasan pnpm lint, pnpm typecheck, pnpm test y pnpm format:check, y pnpm build antes de abrir el PR.</t>
+  </si>
+  <si>
+    <t>La historia se prueba a mano en la aplicación, contra la base local en Docker.</t>
+  </si>
+  <si>
+    <t>Tablero</t>
+  </si>
+  <si>
+    <t>La historia queda en Done en GitHub Projects, con su sprint y sus puntos.</t>
   </si>
 </sst>
 </file>
@@ -962,15 +844,6 @@
     </font>
     <font>
       <b/>
-      <i/>
-      <sz val="16"/>
-      <color rgb="FFC00000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="14"/>
       <name val="Helvetica Neue"/>
       <family val="2"/>
@@ -979,6 +852,13 @@
       <sz val="14"/>
       <name val="Helvetica Neue"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="48">
@@ -1854,7 +1734,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="152">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1988,9 +1868,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="34" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -2267,6 +2147,7 @@
     <xf numFmtId="0" fontId="14" fillId="43" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="47">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -19990,10 +19871,10 @@
         <v>12</v>
       </c>
       <c r="B3" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C3" s="65" t="s">
-        <v>132</v>
+        <v>88</v>
       </c>
       <c r="D3" s="66"/>
       <c r="E3" s="64" t="s">
@@ -20037,10 +19918,10 @@
         <v>15</v>
       </c>
       <c r="B4" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C4" s="65" t="s">
-        <v>133</v>
+        <v>89</v>
       </c>
       <c r="D4" s="66"/>
       <c r="E4" s="64" t="s">
@@ -20084,10 +19965,10 @@
         <v>16</v>
       </c>
       <c r="B5" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C5" s="65" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="D5" s="66"/>
       <c r="E5" s="64" t="s">
@@ -20131,10 +20012,10 @@
         <v>18</v>
       </c>
       <c r="B6" s="65" t="s">
-        <v>135</v>
+        <v>91</v>
       </c>
       <c r="C6" s="65" t="s">
-        <v>136</v>
+        <v>92</v>
       </c>
       <c r="D6" s="66"/>
       <c r="E6" s="64" t="s">
@@ -20178,10 +20059,10 @@
         <v>22</v>
       </c>
       <c r="B7" s="65" t="s">
-        <v>137</v>
+        <v>93</v>
       </c>
       <c r="C7" s="65" t="s">
-        <v>138</v>
+        <v>94</v>
       </c>
       <c r="D7" s="66"/>
       <c r="E7" s="64" t="s">
@@ -20225,10 +20106,10 @@
         <v>28</v>
       </c>
       <c r="B8" s="65" t="s">
-        <v>137</v>
+        <v>93</v>
       </c>
       <c r="C8" s="65" t="s">
-        <v>139</v>
+        <v>95</v>
       </c>
       <c r="D8" s="66"/>
       <c r="E8" s="64" t="s">
@@ -20272,17 +20153,17 @@
         <v>35</v>
       </c>
       <c r="B9" s="65" t="s">
-        <v>140</v>
+        <v>96</v>
       </c>
       <c r="C9" s="65" t="s">
-        <v>141</v>
+        <v>97</v>
       </c>
       <c r="D9" s="66"/>
       <c r="E9" s="64" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="64" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="G9" s="64">
         <v>0</v>
@@ -20319,10 +20200,10 @@
         <v>43</v>
       </c>
       <c r="B10" s="65" t="s">
-        <v>137</v>
+        <v>93</v>
       </c>
       <c r="C10" s="65" t="s">
-        <v>142</v>
+        <v>98</v>
       </c>
       <c r="D10" s="66"/>
       <c r="E10" s="64" t="s">
@@ -20366,10 +20247,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C11" s="65" t="s">
-        <v>143</v>
+        <v>99</v>
       </c>
       <c r="D11" s="66"/>
       <c r="E11" s="64" t="s">
@@ -20413,10 +20294,10 @@
         <v>4</v>
       </c>
       <c r="B12" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C12" s="65" t="s">
-        <v>144</v>
+        <v>100</v>
       </c>
       <c r="D12" s="66"/>
       <c r="E12" s="64" t="s">
@@ -20460,10 +20341,10 @@
         <v>5</v>
       </c>
       <c r="B13" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C13" s="65" t="s">
-        <v>145</v>
+        <v>101</v>
       </c>
       <c r="D13" s="66"/>
       <c r="E13" s="64" t="s">
@@ -20507,10 +20388,10 @@
         <v>6</v>
       </c>
       <c r="B14" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C14" s="65" t="s">
-        <v>146</v>
+        <v>102</v>
       </c>
       <c r="D14" s="66"/>
       <c r="E14" s="64" t="s">
@@ -20554,10 +20435,10 @@
         <v>7</v>
       </c>
       <c r="B15" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C15" s="65" t="s">
-        <v>147</v>
+        <v>103</v>
       </c>
       <c r="D15" s="66"/>
       <c r="E15" s="64" t="s">
@@ -20601,10 +20482,10 @@
         <v>8</v>
       </c>
       <c r="B16" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C16" s="65" t="s">
-        <v>148</v>
+        <v>104</v>
       </c>
       <c r="D16" s="66"/>
       <c r="E16" s="64" t="s">
@@ -20648,10 +20529,10 @@
         <v>9</v>
       </c>
       <c r="B17" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C17" s="65" t="s">
-        <v>149</v>
+        <v>105</v>
       </c>
       <c r="D17" s="66"/>
       <c r="E17" s="64" t="s">
@@ -20695,10 +20576,10 @@
         <v>10</v>
       </c>
       <c r="B18" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C18" s="65" t="s">
-        <v>150</v>
+        <v>106</v>
       </c>
       <c r="D18" s="66"/>
       <c r="E18" s="64" t="s">
@@ -20742,10 +20623,10 @@
         <v>31</v>
       </c>
       <c r="B19" s="65" t="s">
-        <v>137</v>
+        <v>93</v>
       </c>
       <c r="C19" s="65" t="s">
-        <v>151</v>
+        <v>107</v>
       </c>
       <c r="D19" s="66"/>
       <c r="E19" s="64" t="s">
@@ -20789,17 +20670,17 @@
         <v>32</v>
       </c>
       <c r="B20" s="65" t="s">
-        <v>140</v>
+        <v>96</v>
       </c>
       <c r="C20" s="65" t="s">
-        <v>152</v>
+        <v>108</v>
       </c>
       <c r="D20" s="66"/>
       <c r="E20" s="64" t="s">
         <v>23</v>
       </c>
       <c r="F20" s="64" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="G20" s="64">
         <v>0</v>
@@ -20836,17 +20717,17 @@
         <v>33</v>
       </c>
       <c r="B21" s="65" t="s">
-        <v>140</v>
+        <v>96</v>
       </c>
       <c r="C21" s="65" t="s">
-        <v>153</v>
+        <v>109</v>
       </c>
       <c r="D21" s="66"/>
       <c r="E21" s="64" t="s">
         <v>23</v>
       </c>
       <c r="F21" s="64" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="G21" s="64">
         <v>0</v>
@@ -20883,17 +20764,17 @@
         <v>34</v>
       </c>
       <c r="B22" s="65" t="s">
-        <v>140</v>
+        <v>96</v>
       </c>
       <c r="C22" s="65" t="s">
-        <v>154</v>
+        <v>110</v>
       </c>
       <c r="D22" s="66"/>
       <c r="E22" s="64" t="s">
         <v>23</v>
       </c>
       <c r="F22" s="64" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="G22" s="64">
         <v>0</v>
@@ -20930,17 +20811,17 @@
         <v>36</v>
       </c>
       <c r="B23" s="65" t="s">
-        <v>140</v>
+        <v>96</v>
       </c>
       <c r="C23" s="65" t="s">
-        <v>155</v>
+        <v>111</v>
       </c>
       <c r="D23" s="66"/>
       <c r="E23" s="64" t="s">
         <v>23</v>
       </c>
       <c r="F23" s="64" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="G23" s="64">
         <v>0</v>
@@ -25131,7 +25012,7 @@
   <sheetData>
     <row r="2" spans="2:19">
       <c r="B2" s="12" t="s">
-        <v>126</v>
+        <v>82</v>
       </c>
       <c r="C2" s="105" t="s">
         <v>30</v>
@@ -25142,7 +25023,7 @@
     </row>
     <row r="4" spans="2:19" ht="16">
       <c r="B4" s="140" t="s">
-        <v>125</v>
+        <v>81</v>
       </c>
       <c r="C4" s="141"/>
       <c r="D4" s="141"/>
@@ -25608,7 +25489,7 @@
         <v>38</v>
       </c>
       <c r="E2" s="127" t="s">
-        <v>127</v>
+        <v>83</v>
       </c>
       <c r="F2" s="128" t="s">
         <v>39</v>
@@ -25778,13 +25659,13 @@
     </row>
     <row r="18" spans="3:4">
       <c r="C18" s="143" t="s">
-        <v>122</v>
+        <v>78</v>
       </c>
       <c r="D18" s="143"/>
     </row>
     <row r="19" spans="3:4">
       <c r="C19" s="3" t="s">
-        <v>123</v>
+        <v>79</v>
       </c>
       <c r="D19" s="50">
         <f>'Cone of Uncertainty'!E8-'Cone of Uncertainty'!E4</f>
@@ -25801,7 +25682,7 @@
     </row>
     <row r="21" spans="3:4" ht="16">
       <c r="C21" s="21" t="s">
-        <v>124</v>
+        <v>80</v>
       </c>
       <c r="D21" s="19">
         <v>2</v>
@@ -26075,7 +25956,7 @@
         <v>1</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>156</v>
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="2:3">
@@ -26083,7 +25964,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>157</v>
+        <v>113</v>
       </c>
     </row>
     <row r="5" spans="2:3">
@@ -26091,7 +25972,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>158</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="2:3">
@@ -26099,7 +25980,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>159</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="2:3">
@@ -26107,7 +25988,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>160</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" spans="2:3">
@@ -26115,7 +25996,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>161</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" spans="2:3">
@@ -26123,7 +26004,7 @@
         <v>7</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>162</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" spans="2:3">
@@ -26131,7 +26012,7 @@
         <v>8</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>163</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="2:3">
@@ -26174,7 +26055,7 @@
   <sheetData>
     <row r="1" spans="1:20" ht="19.25" customHeight="1">
       <c r="A1" s="149" t="s">
-        <v>54</v>
+        <v>120</v>
       </c>
       <c r="B1" s="149"/>
       <c r="C1" s="149"/>
@@ -26220,218 +26101,159 @@
     </row>
     <row r="4" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="A4" s="56" t="s">
-        <v>55</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B5" s="58" t="s">
-        <v>56</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B6" s="58" t="s">
-        <v>57</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B7" s="58" t="s">
-        <v>58</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:20" s="57" customFormat="1" ht="18">
-      <c r="B8" s="58" t="s">
-        <v>59</v>
-      </c>
+      <c r="A8" s="152" t="s">
+        <v>125</v>
+      </c>
+      <c r="B8" s="58"/>
     </row>
     <row r="9" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B9" s="58" t="s">
-        <v>60</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B10" s="58" t="s">
-        <v>61</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:20" s="57" customFormat="1" ht="18">
-      <c r="B11" s="58" t="s">
-        <v>62</v>
-      </c>
+      <c r="A11" s="152" t="s">
+        <v>128</v>
+      </c>
+      <c r="B11" s="58"/>
     </row>
     <row r="12" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B12" s="58" t="s">
-        <v>63</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B13" s="58" t="s">
-        <v>64</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:20" s="57" customFormat="1" ht="18">
-      <c r="B14" s="58" t="s">
-        <v>65</v>
-      </c>
+      <c r="A14" s="152" t="s">
+        <v>131</v>
+      </c>
+      <c r="B14" s="58"/>
     </row>
     <row r="15" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B15" s="58" t="s">
-        <v>66</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:20" s="57" customFormat="1" ht="18">
-      <c r="A16" s="56" t="s">
-        <v>67</v>
-      </c>
+      <c r="A16" s="56"/>
     </row>
     <row r="17" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B17" s="58" t="s">
-        <v>68</v>
-      </c>
+      <c r="B17" s="58"/>
     </row>
     <row r="18" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B18" s="58" t="s">
-        <v>69</v>
-      </c>
+      <c r="B18" s="58"/>
     </row>
     <row r="19" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="A19" s="56" t="s">
-        <v>70</v>
-      </c>
+      <c r="A19" s="56"/>
     </row>
     <row r="20" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B20" s="58" t="s">
-        <v>71</v>
-      </c>
+      <c r="B20" s="58"/>
     </row>
     <row r="21" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B21" s="58" t="s">
-        <v>72</v>
-      </c>
+      <c r="B21" s="58"/>
     </row>
     <row r="22" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B22" s="58" t="s">
-        <v>73</v>
-      </c>
+      <c r="B22" s="58"/>
     </row>
     <row r="23" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B23" s="58" t="s">
-        <v>74</v>
-      </c>
+      <c r="B23" s="58"/>
     </row>
     <row r="24" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B24" s="58" t="s">
-        <v>75</v>
-      </c>
+      <c r="B24" s="58"/>
     </row>
     <row r="25" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B25" s="58" t="s">
-        <v>76</v>
-      </c>
+      <c r="B25" s="58"/>
     </row>
     <row r="26" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B26" s="58" t="s">
-        <v>77</v>
-      </c>
+      <c r="B26" s="58"/>
     </row>
     <row r="27" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B27" s="58" t="s">
-        <v>78</v>
-      </c>
+      <c r="B27" s="58"/>
     </row>
     <row r="28" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B28" s="58" t="s">
-        <v>79</v>
-      </c>
+      <c r="B28" s="58"/>
     </row>
     <row r="29" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B29" s="58" t="s">
-        <v>80</v>
-      </c>
+      <c r="B29" s="58"/>
     </row>
     <row r="30" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B30" s="58" t="s">
-        <v>81</v>
-      </c>
+      <c r="B30" s="58"/>
     </row>
     <row r="31" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B31" s="58" t="s">
-        <v>82</v>
-      </c>
+      <c r="B31" s="58"/>
     </row>
     <row r="32" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B32" s="58" t="s">
-        <v>83</v>
-      </c>
+      <c r="B32" s="58"/>
     </row>
     <row r="33" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B33" s="58" t="s">
-        <v>84</v>
-      </c>
+      <c r="B33" s="58"/>
     </row>
     <row r="34" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="A34" s="56" t="s">
-        <v>85</v>
-      </c>
+      <c r="A34" s="56"/>
     </row>
     <row r="35" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B35" s="58" t="s">
-        <v>86</v>
-      </c>
+      <c r="B35" s="58"/>
     </row>
     <row r="36" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B36" s="58" t="s">
-        <v>87</v>
-      </c>
+      <c r="B36" s="58"/>
     </row>
     <row r="37" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B37" s="58" t="s">
-        <v>88</v>
-      </c>
+      <c r="B37" s="58"/>
     </row>
     <row r="38" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="A38" s="56" t="s">
-        <v>89</v>
-      </c>
+      <c r="A38" s="56"/>
     </row>
     <row r="39" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B39" s="58" t="s">
-        <v>90</v>
-      </c>
+      <c r="B39" s="58"/>
     </row>
     <row r="40" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B40" s="58" t="s">
-        <v>91</v>
-      </c>
+      <c r="B40" s="58"/>
     </row>
     <row r="41" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B41" s="58" t="s">
-        <v>92</v>
-      </c>
+      <c r="B41" s="58"/>
     </row>
     <row r="42" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B42" s="58" t="s">
-        <v>93</v>
-      </c>
+      <c r="B42" s="58"/>
     </row>
     <row r="43" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B43" s="58" t="s">
-        <v>94</v>
-      </c>
+      <c r="B43" s="58"/>
     </row>
     <row r="44" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B44" s="58" t="s">
-        <v>95</v>
-      </c>
+      <c r="B44" s="58"/>
     </row>
     <row r="45" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B45" s="58" t="s">
-        <v>96</v>
-      </c>
+      <c r="B45" s="58"/>
     </row>
     <row r="46" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B46" s="58" t="s">
-        <v>97</v>
-      </c>
+      <c r="B46" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -26465,100 +26287,100 @@
   <sheetData>
     <row r="2" spans="2:4">
       <c r="B2" s="134" t="s">
-        <v>98</v>
+        <v>54</v>
       </c>
       <c r="C2" s="135"/>
       <c r="D2" s="136"/>
     </row>
     <row r="3" spans="2:4" ht="14.25" customHeight="1">
       <c r="B3" s="116" t="s">
-        <v>99</v>
+        <v>55</v>
       </c>
       <c r="C3" s="116" t="s">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="D3" s="116" t="s">
-        <v>101</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="2:4">
       <c r="B4" s="3" t="s">
-        <v>128</v>
+        <v>84</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="D4" s="3"/>
     </row>
     <row r="5" spans="2:4">
       <c r="B5" s="3" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>103</v>
+        <v>59</v>
       </c>
       <c r="D5" s="3"/>
     </row>
     <row r="6" spans="2:4">
       <c r="B6" s="3" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>104</v>
+        <v>60</v>
       </c>
       <c r="D6" s="3"/>
     </row>
     <row r="7" spans="2:4">
       <c r="B7" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>104</v>
+        <v>60</v>
       </c>
       <c r="D7" s="3"/>
     </row>
     <row r="8" spans="2:4">
       <c r="B8" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>105</v>
+        <v>61</v>
       </c>
       <c r="D8" s="3"/>
     </row>
     <row r="9" spans="2:4">
       <c r="B9" s="3" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="D9" s="3"/>
     </row>
     <row r="10" spans="2:4">
       <c r="B10" s="3" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>107</v>
+        <v>63</v>
       </c>
       <c r="D10" s="27"/>
     </row>
     <row r="11" spans="2:4">
       <c r="B11" s="3" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>108</v>
+        <v>64</v>
       </c>
       <c r="D11" s="27"/>
     </row>
     <row r="12" spans="2:4">
       <c r="B12" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>109</v>
+        <v>65</v>
       </c>
       <c r="D12" s="27"/>
     </row>
@@ -26633,39 +26455,39 @@
     <row r="3" spans="2:20" ht="46.5" customHeight="1">
       <c r="B3" s="2"/>
       <c r="C3" s="116" t="s">
-        <v>110</v>
+        <v>66</v>
       </c>
       <c r="D3" s="115" t="s">
-        <v>111</v>
+        <v>67</v>
       </c>
       <c r="E3" s="115" t="s">
-        <v>112</v>
+        <v>68</v>
       </c>
       <c r="F3" s="115" t="s">
-        <v>113</v>
+        <v>69</v>
       </c>
       <c r="G3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="151" t="s">
-        <v>114</v>
+        <v>70</v>
       </c>
       <c r="K3" s="151"/>
       <c r="L3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="115" t="s">
-        <v>115</v>
+        <v>71</v>
       </c>
       <c r="P3" s="2"/>
       <c r="R3" s="2"/>
       <c r="S3" s="116" t="s">
-        <v>117</v>
+        <v>73</v>
       </c>
       <c r="T3" s="2"/>
     </row>
     <row r="4" spans="2:20">
       <c r="B4" s="2"/>
       <c r="C4" s="3" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="D4" s="11">
         <v>0</v>
@@ -26679,7 +26501,7 @@
       <c r="G4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="3" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="K4" s="1">
         <v>0</v>
@@ -26898,34 +26720,34 @@
     <row r="12" spans="2:20" ht="44.25" customHeight="1">
       <c r="B12" s="2"/>
       <c r="C12" s="116" t="s">
-        <v>110</v>
+        <v>66</v>
       </c>
       <c r="D12" s="115" t="s">
-        <v>119</v>
+        <v>75</v>
       </c>
       <c r="E12" s="115" t="s">
-        <v>120</v>
+        <v>76</v>
       </c>
       <c r="F12" s="115" t="s">
-        <v>121</v>
+        <v>77</v>
       </c>
       <c r="G12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="151" t="s">
-        <v>114</v>
+        <v>70</v>
       </c>
       <c r="K12" s="151"/>
       <c r="L12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="115" t="s">
-        <v>116</v>
+        <v>72</v>
       </c>
       <c r="P12" s="2"/>
     </row>
     <row r="13" spans="2:20">
       <c r="B13" s="2"/>
       <c r="C13" s="3" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="D13" s="11">
         <v>0</v>
@@ -26942,7 +26764,7 @@
         <v>0</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="L13" s="2"/>
       <c r="N13" s="2"/>
@@ -27187,6 +27009,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006DEE37CDC9AEA44CBD8F091652A6C5E4" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9de09e14d18b2e0769f00e11c33b035a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7bb3299b-b075-41c7-bb54-99fc85b15d4f" xmlns:ns3="08caf6cd-a550-4dce-b6c8-fe9b0e6bc4e3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="81a6a9a579b993e4978c34f4e71e25a5" ns2:_="" ns3:_="">
     <xsd:import namespace="7bb3299b-b075-41c7-bb54-99fc85b15d4f"/>
@@ -27397,12 +27225,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -27413,6 +27235,15 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF49F70C-261C-4E13-A8B5-F2B201AA0A03}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D916E78-7E6F-4E04-B4AA-CEC365547DDB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -27431,15 +27262,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF49F70C-261C-4E13-A8B5-F2B201AA0A03}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1010AAFC-6E8A-4F4B-91D1-B1DB8DD7131E}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
docs(entrega-2): assumptions, definition of done and checklist sync (#57)
* docs(entrega-2): state the assumptions behind the cone

Velocity, team size, sample vacancies, no LinkedIn API, local deployment, and why Operate and Technical Items are zero.

* docs(entrega-2): replace the template's definition of done with the team's

Acceptance criteria, issue and branch, domain rules tested in core, review requested on the PR, the five checks green, and the board updated.

* docs(entrega-2): drop the duplicated retrospective label

* docs(entrega-2): sync the checklist with the retrospective and diagrams on main

The class diagram is not in the repository yet, so it is unticked; the retrospective technique and actions are.
</commit_message>
<xml_diff>
--- a/docs/deliverables/delivery-2/document/Entrega2_Template_HistoriasUsuario.xlsx
+++ b/docs/deliverables/delivery-2/document/Entrega2_Template_HistoriasUsuario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pablo/Library/Containers/com.microsoft.Excel/Data/tmp/ml/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42DD1CE2-21C4-7745-B942-0C911EDD63D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D64F0FD-42B8-6143-A42D-7126D1496034}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4880" yWindow="600" windowWidth="34500" windowHeight="22820" tabRatio="677" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -193,7 +193,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="133">
   <si>
     <t>Features backlog</t>
   </si>
@@ -360,163 +360,6 @@
   </si>
   <si>
     <t>Assumptions</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">This template uses an average velocity (Story Points) to calculate the cone of uncertainty (duration interval). For that to be valid you'll need the estimation team to allign on what "done" means and what activities are included. The below is an </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="16"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>example</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="16"/>
-        <color rgb="FFC00000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> as a starting points and should be tailored case-by-case</t>
-    </r>
-  </si>
-  <si>
-    <t>Development</t>
-  </si>
-  <si>
-    <t>Technical Implementation Plan confirmed with architects/TL [if needed].</t>
-  </si>
-  <si>
-    <t>Code written and tested locally.</t>
-  </si>
-  <si>
-    <t>Unit Tests developed for Back-end ( 80% code coverage) and Front-end ( 60% code coverage).</t>
-  </si>
-  <si>
-    <t>Code reviewed and approved by at least one mandatory approval.</t>
-  </si>
-  <si>
-    <t>Documentation of model/controllers/sequence diagrams [if needed].</t>
-  </si>
-  <si>
-    <t>IDs for FE elements ( where needed). - checked on code review &amp; testing.</t>
-  </si>
-  <si>
-    <t>Configuration check - (if needed ) added in release notes.</t>
-  </si>
-  <si>
-    <t>Release notes updated.</t>
-  </si>
-  <si>
-    <t>Sonar execution on review - no critical issues accepted.</t>
-  </si>
-  <si>
-    <t>English labels available in CMS ( if needed).</t>
-  </si>
-  <si>
-    <t>All defects reported by testing fixed.</t>
-  </si>
-  <si>
-    <t>Deployment/Demo</t>
-  </si>
-  <si>
-    <t>Changes deployed successfully to Openshift Director env (no build error + sonar passed successfully )  &gt;= 5 SP (2 days before sprint ends), only bug fixing will be allowed.</t>
-  </si>
-  <si>
-    <t>Deployment freeze also 3 hours before demo.</t>
-  </si>
-  <si>
-    <t>Testing</t>
-  </si>
-  <si>
-    <t>Test cases written in Zephyr.</t>
-  </si>
-  <si>
-    <t>Application tested against the mock layer, including error cases and edge.</t>
-  </si>
-  <si>
-    <t>Manual functional test 100% test coverage on test environment.</t>
-  </si>
-  <si>
-    <t>Manual test (basic and advanced) cases executed and passing.</t>
-  </si>
-  <si>
-    <t>Exploratory testing executed.</t>
-  </si>
-  <si>
-    <t>Testing passed 100% on Test Environment.</t>
-  </si>
-  <si>
-    <t>All issues reported as bugs and linked to the stories.</t>
-  </si>
-  <si>
-    <t>Acceptance criteria fulfilled.</t>
-  </si>
-  <si>
-    <t>Test data is documented.</t>
-  </si>
-  <si>
-    <t>NFR fulfilled.</t>
-  </si>
-  <si>
-    <t>Quality Acceptance.</t>
-  </si>
-  <si>
-    <t>No issues with severity worse than Major.</t>
-  </si>
-  <si>
-    <t>Feature documented in TBD owner.</t>
-  </si>
-  <si>
-    <t>User story is updated with latest information/requirements.</t>
-  </si>
-  <si>
-    <t>Automated testing</t>
-  </si>
-  <si>
-    <t>Automated tests written.</t>
-  </si>
-  <si>
-    <t>Automated tests committed to Git.</t>
-  </si>
-  <si>
-    <t>Automated tests executed and validated.</t>
-  </si>
-  <si>
-    <t>Other considerations</t>
-  </si>
-  <si>
-    <t>(TBD story by story</t>
-  </si>
-  <si>
-    <t>OR add a separate story)</t>
-  </si>
-  <si>
-    <t>*all to be covered with Acceptance criteria.</t>
-  </si>
-  <si>
-    <t>Performance.</t>
-  </si>
-  <si>
-    <t>Security.</t>
-  </si>
-  <si>
-    <t>Error handling.</t>
-  </si>
-  <si>
-    <t>Localization.</t>
-  </si>
-  <si>
-    <t>In-house usability testing.</t>
   </si>
   <si>
     <t>Delivery Team(s) Shape</t>
@@ -692,6 +535,69 @@
   </si>
   <si>
     <t>#36 Logging without sensitive data</t>
+  </si>
+  <si>
+    <t>La velocidad promedio es de 50 puntos por sprint, la que logró el equipo en el Sprint 1.</t>
+  </si>
+  <si>
+    <t>El equipo son dos personas, con la misma disponibilidad en todos los sprints.</t>
+  </si>
+  <si>
+    <t>Los puntos de las historias de la fase Later no cambian al refinarlas.</t>
+  </si>
+  <si>
+    <t>Las vacantes vienen de un conjunto de prueba de 20, no de datos reales de Magneto.</t>
+  </si>
+  <si>
+    <t>No se cuenta con una API de LinkedIn que entregue la experiencia, la educación y las habilidades del perfil.</t>
+  </si>
+  <si>
+    <t>El despliegue local es suficiente para las entregas, como lo permite el reto.</t>
+  </si>
+  <si>
+    <t>Las historias no funcionales (#32 a #36) no se estiman en puntos, así que no entran en el cono.</t>
+  </si>
+  <si>
+    <t>No hay sprints de operación ni de puesta en producción, y el ambiente de desarrollo (Docker y el monorepo) existe desde el Sprint 1. Por eso Operate y Technical Items valen 0.</t>
+  </si>
+  <si>
+    <t>Una historia cuenta como terminada, y suma a la velocidad del cono, solo cuando cumple todo lo de esta hoja.</t>
+  </si>
+  <si>
+    <t>Desarrollo</t>
+  </si>
+  <si>
+    <t>Los criterios de aceptación de la historia se cumplen todos.</t>
+  </si>
+  <si>
+    <t>La historia tiene su issue y su propia rama, creada desde main.</t>
+  </si>
+  <si>
+    <t>Las reglas del dominio viven en packages/core y tienen pruebas; el SQL vive solo en packages/db.</t>
+  </si>
+  <si>
+    <t>Revisión</t>
+  </si>
+  <si>
+    <t>El PR enlaza su issue con Closes #N y pide la revisión del otro integrante.</t>
+  </si>
+  <si>
+    <t>Se integra con squash merge y la rama se borra.</t>
+  </si>
+  <si>
+    <t>Pruebas</t>
+  </si>
+  <si>
+    <t>Pasan pnpm lint, pnpm typecheck, pnpm test y pnpm format:check, y pnpm build antes de abrir el PR.</t>
+  </si>
+  <si>
+    <t>La historia se prueba a mano en la aplicación, contra la base local en Docker.</t>
+  </si>
+  <si>
+    <t>Tablero</t>
+  </si>
+  <si>
+    <t>La historia queda en Done en GitHub Projects, con su sprint y sus puntos.</t>
   </si>
 </sst>
 </file>
@@ -938,15 +844,6 @@
     </font>
     <font>
       <b/>
-      <i/>
-      <sz val="16"/>
-      <color rgb="FFC00000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="14"/>
       <name val="Helvetica Neue"/>
       <family val="2"/>
@@ -955,6 +852,13 @@
       <sz val="14"/>
       <name val="Helvetica Neue"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="48">
@@ -1830,7 +1734,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="152">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1964,9 +1868,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="1" fillId="34" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -2188,6 +2092,15 @@
     <xf numFmtId="2" fontId="18" fillId="44" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="43" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="43" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="43" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="47" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2228,21 +2141,13 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="43" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="43" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="43" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="43" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="47">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2296,6 +2201,38 @@
   <dxfs count="38">
     <dxf>
       <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="9" tint="-0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2328,6 +2265,30 @@
         <bottom style="medium">
           <color theme="0"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.34998626667073579"/>
+        </patternFill>
+      </fill>
+      <border outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
       </border>
     </dxf>
     <dxf>
@@ -2370,6 +2331,30 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="1" tint="0.34998626667073579"/>
+        </patternFill>
+      </fill>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2402,6 +2387,41 @@
         </top>
         <bottom style="medium">
           <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFCA3B41"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
         </bottom>
       </border>
     </dxf>
@@ -2444,6 +2464,41 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF7BE66"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2476,6 +2531,41 @@
         </top>
         <bottom style="medium">
           <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="166" formatCode="0.0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF487B48"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+        <bottom style="thin">
+          <color auto="1"/>
         </bottom>
       </border>
     </dxf>
@@ -2514,6 +2604,24 @@
         <bottom style="medium">
           <color theme="0"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border outline="0">
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
       </border>
     </dxf>
     <dxf>
@@ -2557,42 +2665,16 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
         <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="12"/>
-        <color theme="0"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.34998626667073579"/>
-        </right>
-        <top style="medium">
-          <color theme="0"/>
-        </top>
-        <bottom style="medium">
-          <color theme="0"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -2635,6 +2717,19 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2671,6 +2766,71 @@
           <color theme="0"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </left>
+        <right style="thin">
+          <color theme="0" tint="-0.34998626667073579"/>
+        </right>
+        <top style="medium">
+          <color theme="0"/>
+        </top>
+        <bottom style="medium">
+          <color theme="0"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -2713,6 +2873,19 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2749,6 +2922,19 @@
           <color theme="0"/>
         </bottom>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -2791,6 +2977,19 @@
     </dxf>
     <dxf>
       <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -2827,300 +3026,6 @@
           <color theme="0"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="9" tint="-0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="1" tint="0.34998626667073579"/>
-        </patternFill>
-      </fill>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0.0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFCA3B41"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0.0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFF7BE66"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="166" formatCode="0.0"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF487B48"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="1"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border outline="0">
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -19448,28 +19353,28 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A2:N24" totalsRowCount="1" headerRowDxfId="37" dataDxfId="36" totalsRowDxfId="35" totalsRowBorderDxfId="34">
   <autoFilter ref="A2:N23" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" totalsRowLabel="Total" dataDxfId="33" totalsRowDxfId="13"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Capability" dataDxfId="32" totalsRowDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Backlog Item _x000a_(Feature or Story)" dataDxfId="31" totalsRowDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Comments" dataDxfId="30" totalsRowDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase" dataDxfId="29" totalsRowDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Tshirt Sizing" dataDxfId="28" totalsRowDxfId="8"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Story Points" dataDxfId="27" totalsRowDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Business Uncertainty" dataDxfId="26" totalsRowDxfId="6"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Technical Complexity" dataDxfId="25" totalsRowDxfId="5"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="BEST CASE" totalsRowFunction="sum" dataDxfId="24" totalsRowDxfId="4">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" totalsRowLabel="Total" dataDxfId="33" totalsRowDxfId="32"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Capability" dataDxfId="31" totalsRowDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Backlog Item _x000a_(Feature or Story)" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Comments" dataDxfId="27" totalsRowDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Phase" dataDxfId="25" totalsRowDxfId="24"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Tshirt Sizing" dataDxfId="23" totalsRowDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Story Points" dataDxfId="21" totalsRowDxfId="20"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Business Uncertainty" dataDxfId="19" totalsRowDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Technical Complexity" dataDxfId="17" totalsRowDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="BEST CASE" totalsRowFunction="sum" dataDxfId="15" totalsRowDxfId="14">
       <calculatedColumnFormula>IFERROR((K3-K3*M3),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="MOST LIKELY" totalsRowFunction="sum" dataDxfId="23" totalsRowDxfId="3">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="MOST LIKELY" totalsRowFunction="sum" dataDxfId="13" totalsRowDxfId="12">
       <calculatedColumnFormula>IFERROR((IF(ISBLANK(G3),VLOOKUP(F3,lst_TShirt_2_SP_Avg,2,FALSE),G3)),0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="WORST CASE" totalsRowFunction="sum" dataDxfId="22" totalsRowDxfId="2">
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="WORST CASE" totalsRowFunction="sum" dataDxfId="11" totalsRowDxfId="10">
       <calculatedColumnFormula>K3+K3*M3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="CONE of Uncertainty" dataDxfId="21" totalsRowDxfId="1">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="CONE of Uncertainty" dataDxfId="9" totalsRowDxfId="8">
       <calculatedColumnFormula>IF(H3="Low",VLOOKUP(N3,lst_tshirt_bu,2,FALSE),IF(H3="Medium",VLOOKUP(N3,lst_tshirt_bu,3,FALSE),IF(H3="High",VLOOKUP(N3,lst_tshirt_bu,4,FALSE),0))) + IF(I3="Low",VLOOKUP(N3,lst_tshirt_tc,2,FALSE),IF(I3="Medium",VLOOKUP(N3,lst_tshirt_tc,3,FALSE),IF(I3="High",VLOOKUP(N3,lst_tshirt_tc,4,FALSE),0)))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Tshirt Size for Cone Calc" dataDxfId="20" totalsRowDxfId="0">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Tshirt Size for Cone Calc" dataDxfId="7" totalsRowDxfId="6">
       <calculatedColumnFormula>IF(ISBLANK(G3),F3,VLOOKUP(G3,lst_SP_to_TShirt,2,FALSE))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -19827,22 +19732,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:87" ht="18" customHeight="1" thickBot="1">
-      <c r="A1" s="134" t="s">
+      <c r="A1" s="137" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="135"/>
-      <c r="C1" s="135"/>
-      <c r="D1" s="135"/>
-      <c r="E1" s="135"/>
-      <c r="F1" s="135"/>
-      <c r="G1" s="135"/>
-      <c r="H1" s="135"/>
-      <c r="I1" s="135"/>
-      <c r="J1" s="135"/>
-      <c r="K1" s="135"/>
-      <c r="L1" s="135"/>
-      <c r="M1" s="135"/>
-      <c r="N1" s="136"/>
+      <c r="B1" s="138"/>
+      <c r="C1" s="138"/>
+      <c r="D1" s="138"/>
+      <c r="E1" s="138"/>
+      <c r="F1" s="138"/>
+      <c r="G1" s="138"/>
+      <c r="H1" s="138"/>
+      <c r="I1" s="138"/>
+      <c r="J1" s="138"/>
+      <c r="K1" s="138"/>
+      <c r="L1" s="138"/>
+      <c r="M1" s="138"/>
+      <c r="N1" s="139"/>
     </row>
     <row r="2" spans="1:87" s="14" customFormat="1" ht="51">
       <c r="A2" s="23" t="s">
@@ -19966,10 +19871,10 @@
         <v>12</v>
       </c>
       <c r="B3" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C3" s="65" t="s">
-        <v>132</v>
+        <v>88</v>
       </c>
       <c r="D3" s="66"/>
       <c r="E3" s="64" t="s">
@@ -20013,10 +19918,10 @@
         <v>15</v>
       </c>
       <c r="B4" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C4" s="65" t="s">
-        <v>133</v>
+        <v>89</v>
       </c>
       <c r="D4" s="66"/>
       <c r="E4" s="64" t="s">
@@ -20060,10 +19965,10 @@
         <v>16</v>
       </c>
       <c r="B5" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C5" s="65" t="s">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="D5" s="66"/>
       <c r="E5" s="64" t="s">
@@ -20107,10 +20012,10 @@
         <v>18</v>
       </c>
       <c r="B6" s="65" t="s">
-        <v>135</v>
+        <v>91</v>
       </c>
       <c r="C6" s="65" t="s">
-        <v>136</v>
+        <v>92</v>
       </c>
       <c r="D6" s="66"/>
       <c r="E6" s="64" t="s">
@@ -20154,10 +20059,10 @@
         <v>22</v>
       </c>
       <c r="B7" s="65" t="s">
-        <v>137</v>
+        <v>93</v>
       </c>
       <c r="C7" s="65" t="s">
-        <v>138</v>
+        <v>94</v>
       </c>
       <c r="D7" s="66"/>
       <c r="E7" s="64" t="s">
@@ -20201,10 +20106,10 @@
         <v>28</v>
       </c>
       <c r="B8" s="65" t="s">
-        <v>137</v>
+        <v>93</v>
       </c>
       <c r="C8" s="65" t="s">
-        <v>139</v>
+        <v>95</v>
       </c>
       <c r="D8" s="66"/>
       <c r="E8" s="64" t="s">
@@ -20248,17 +20153,17 @@
         <v>35</v>
       </c>
       <c r="B9" s="65" t="s">
-        <v>140</v>
+        <v>96</v>
       </c>
       <c r="C9" s="65" t="s">
-        <v>141</v>
+        <v>97</v>
       </c>
       <c r="D9" s="66"/>
       <c r="E9" s="64" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="64" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="G9" s="64">
         <v>0</v>
@@ -20295,10 +20200,10 @@
         <v>43</v>
       </c>
       <c r="B10" s="65" t="s">
-        <v>137</v>
+        <v>93</v>
       </c>
       <c r="C10" s="65" t="s">
-        <v>142</v>
+        <v>98</v>
       </c>
       <c r="D10" s="66"/>
       <c r="E10" s="64" t="s">
@@ -20342,10 +20247,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C11" s="65" t="s">
-        <v>143</v>
+        <v>99</v>
       </c>
       <c r="D11" s="66"/>
       <c r="E11" s="64" t="s">
@@ -20389,10 +20294,10 @@
         <v>4</v>
       </c>
       <c r="B12" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C12" s="65" t="s">
-        <v>144</v>
+        <v>100</v>
       </c>
       <c r="D12" s="66"/>
       <c r="E12" s="64" t="s">
@@ -20436,10 +20341,10 @@
         <v>5</v>
       </c>
       <c r="B13" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C13" s="65" t="s">
-        <v>145</v>
+        <v>101</v>
       </c>
       <c r="D13" s="66"/>
       <c r="E13" s="64" t="s">
@@ -20483,10 +20388,10 @@
         <v>6</v>
       </c>
       <c r="B14" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C14" s="65" t="s">
-        <v>146</v>
+        <v>102</v>
       </c>
       <c r="D14" s="66"/>
       <c r="E14" s="64" t="s">
@@ -20530,10 +20435,10 @@
         <v>7</v>
       </c>
       <c r="B15" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C15" s="65" t="s">
-        <v>147</v>
+        <v>103</v>
       </c>
       <c r="D15" s="66"/>
       <c r="E15" s="64" t="s">
@@ -20577,10 +20482,10 @@
         <v>8</v>
       </c>
       <c r="B16" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C16" s="65" t="s">
-        <v>148</v>
+        <v>104</v>
       </c>
       <c r="D16" s="66"/>
       <c r="E16" s="64" t="s">
@@ -20624,10 +20529,10 @@
         <v>9</v>
       </c>
       <c r="B17" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C17" s="65" t="s">
-        <v>149</v>
+        <v>105</v>
       </c>
       <c r="D17" s="66"/>
       <c r="E17" s="64" t="s">
@@ -20671,10 +20576,10 @@
         <v>10</v>
       </c>
       <c r="B18" s="65" t="s">
-        <v>131</v>
+        <v>87</v>
       </c>
       <c r="C18" s="65" t="s">
-        <v>150</v>
+        <v>106</v>
       </c>
       <c r="D18" s="66"/>
       <c r="E18" s="64" t="s">
@@ -20718,10 +20623,10 @@
         <v>31</v>
       </c>
       <c r="B19" s="65" t="s">
-        <v>137</v>
+        <v>93</v>
       </c>
       <c r="C19" s="65" t="s">
-        <v>151</v>
+        <v>107</v>
       </c>
       <c r="D19" s="66"/>
       <c r="E19" s="64" t="s">
@@ -20765,17 +20670,17 @@
         <v>32</v>
       </c>
       <c r="B20" s="65" t="s">
-        <v>140</v>
+        <v>96</v>
       </c>
       <c r="C20" s="65" t="s">
-        <v>152</v>
+        <v>108</v>
       </c>
       <c r="D20" s="66"/>
       <c r="E20" s="64" t="s">
         <v>23</v>
       </c>
       <c r="F20" s="64" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="G20" s="64">
         <v>0</v>
@@ -20812,17 +20717,17 @@
         <v>33</v>
       </c>
       <c r="B21" s="65" t="s">
-        <v>140</v>
+        <v>96</v>
       </c>
       <c r="C21" s="65" t="s">
-        <v>153</v>
+        <v>109</v>
       </c>
       <c r="D21" s="66"/>
       <c r="E21" s="64" t="s">
         <v>23</v>
       </c>
       <c r="F21" s="64" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="G21" s="64">
         <v>0</v>
@@ -20859,17 +20764,17 @@
         <v>34</v>
       </c>
       <c r="B22" s="65" t="s">
-        <v>140</v>
+        <v>96</v>
       </c>
       <c r="C22" s="65" t="s">
-        <v>154</v>
+        <v>110</v>
       </c>
       <c r="D22" s="66"/>
       <c r="E22" s="64" t="s">
         <v>23</v>
       </c>
       <c r="F22" s="64" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="G22" s="64">
         <v>0</v>
@@ -20906,17 +20811,17 @@
         <v>36</v>
       </c>
       <c r="B23" s="65" t="s">
-        <v>140</v>
+        <v>96</v>
       </c>
       <c r="C23" s="65" t="s">
-        <v>155</v>
+        <v>111</v>
       </c>
       <c r="D23" s="66"/>
       <c r="E23" s="64" t="s">
         <v>23</v>
       </c>
       <c r="F23" s="64" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="G23" s="64">
         <v>0</v>
@@ -24999,23 +24904,23 @@
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <conditionalFormatting sqref="A3:D23">
-    <cfRule type="expression" dxfId="19" priority="1">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>COUNTBLANK($F3:$G3)=2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A25:M26 H2:I24 N26 O28:Q419 I27:N417">
-    <cfRule type="cellIs" dxfId="18" priority="2" operator="equal">
+  <conditionalFormatting sqref="H2:I24 A25:M26 N26 I27:N417 O28:Q419">
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
       <formula>"High"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="17" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"Medium"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:L2 J24:L24 H27:I1048576">
-    <cfRule type="cellIs" dxfId="16" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="6" operator="equal">
       <formula>"High"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="7" operator="equal">
       <formula>"Medium"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25034,7 +24939,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N3:N23">
-    <cfRule type="expression" dxfId="14" priority="4">
+    <cfRule type="expression" dxfId="0" priority="4">
       <formula>N3&lt;&gt;F3</formula>
     </cfRule>
   </conditionalFormatting>
@@ -25107,7 +25012,7 @@
   <sheetData>
     <row r="2" spans="2:19">
       <c r="B2" s="12" t="s">
-        <v>126</v>
+        <v>82</v>
       </c>
       <c r="C2" s="105" t="s">
         <v>30</v>
@@ -25117,28 +25022,28 @@
       <c r="C3" s="105"/>
     </row>
     <row r="4" spans="2:19" ht="16">
-      <c r="B4" s="137" t="s">
-        <v>125</v>
-      </c>
-      <c r="C4" s="138"/>
-      <c r="D4" s="138"/>
-      <c r="E4" s="138"/>
-      <c r="F4" s="138"/>
-      <c r="G4" s="139"/>
-      <c r="I4" s="137" t="s">
+      <c r="B4" s="140" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4" s="141"/>
+      <c r="D4" s="141"/>
+      <c r="E4" s="141"/>
+      <c r="F4" s="141"/>
+      <c r="G4" s="142"/>
+      <c r="I4" s="140" t="s">
         <v>28</v>
       </c>
-      <c r="J4" s="138"/>
-      <c r="K4" s="138"/>
-      <c r="L4" s="138"/>
-      <c r="M4" s="138"/>
-      <c r="O4" s="137" t="s">
+      <c r="J4" s="141"/>
+      <c r="K4" s="141"/>
+      <c r="L4" s="141"/>
+      <c r="M4" s="141"/>
+      <c r="O4" s="140" t="s">
         <v>29</v>
       </c>
-      <c r="P4" s="138"/>
-      <c r="Q4" s="138"/>
-      <c r="R4" s="138"/>
-      <c r="S4" s="138"/>
+      <c r="P4" s="141"/>
+      <c r="Q4" s="141"/>
+      <c r="R4" s="141"/>
+      <c r="S4" s="141"/>
     </row>
     <row r="5" spans="2:19" ht="51">
       <c r="B5" s="26" t="s">
@@ -25584,14 +25489,14 @@
         <v>38</v>
       </c>
       <c r="E2" s="127" t="s">
-        <v>127</v>
+        <v>83</v>
       </c>
       <c r="F2" s="128" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="3" spans="2:25" ht="0.75" customHeight="1">
-      <c r="C3" s="141" t="s">
+      <c r="C3" s="144" t="s">
         <v>40</v>
       </c>
       <c r="D3" s="117">
@@ -25608,7 +25513,7 @@
       <c r="U3" s="4"/>
     </row>
     <row r="4" spans="2:25" ht="16.25" customHeight="1">
-      <c r="C4" s="141"/>
+      <c r="C4" s="144"/>
       <c r="D4" s="117">
         <f>ROUNDUP(Table1[[#Totals],[BEST CASE]]/avgVelocity,0) + D14 +D15</f>
         <v>1</v>
@@ -25623,7 +25528,7 @@
       </c>
     </row>
     <row r="5" spans="2:25" ht="0.75" customHeight="1">
-      <c r="C5" s="142" t="s">
+      <c r="C5" s="145" t="s">
         <v>41</v>
       </c>
       <c r="D5" s="118">
@@ -25637,7 +25542,7 @@
       </c>
     </row>
     <row r="6" spans="2:25" ht="13.5" customHeight="1">
-      <c r="C6" s="142"/>
+      <c r="C6" s="145"/>
       <c r="D6" s="118">
         <f>ROUNDUP(Table1[[#Totals],[MOST LIKELY]]/avgVelocity,0) + D14 +D15</f>
         <v>2</v>
@@ -25652,7 +25557,7 @@
       </c>
     </row>
     <row r="7" spans="2:25" ht="15" hidden="1" customHeight="1">
-      <c r="C7" s="143" t="s">
+      <c r="C7" s="146" t="s">
         <v>42</v>
       </c>
       <c r="D7" s="119">
@@ -25666,7 +25571,7 @@
       </c>
     </row>
     <row r="8" spans="2:25">
-      <c r="C8" s="143"/>
+      <c r="C8" s="146"/>
       <c r="D8" s="119">
         <f>ROUNDUP(Table1[[#Totals],[WORST CASE]]/avgVelocity,0)  + D14 +D15</f>
         <v>2</v>
@@ -25681,7 +25586,7 @@
       </c>
     </row>
     <row r="9" spans="2:25" ht="0.75" customHeight="1">
-      <c r="C9" s="144" t="s">
+      <c r="C9" s="147" t="s">
         <v>43</v>
       </c>
       <c r="D9" s="120">
@@ -25696,7 +25601,7 @@
       </c>
     </row>
     <row r="10" spans="2:25" ht="16" thickBot="1">
-      <c r="C10" s="145"/>
+      <c r="C10" s="148"/>
       <c r="D10" s="133">
         <f>ROUNDUP(Table1[[#Totals],[MOST LIKELY]]/avgVelocity + 'Cone of Uncertainty'!D21,0)</f>
         <v>4</v>
@@ -25753,14 +25658,14 @@
       <c r="B16" s="55"/>
     </row>
     <row r="18" spans="3:4">
-      <c r="C18" s="140" t="s">
-        <v>122</v>
-      </c>
-      <c r="D18" s="140"/>
+      <c r="C18" s="143" t="s">
+        <v>78</v>
+      </c>
+      <c r="D18" s="143"/>
     </row>
     <row r="19" spans="3:4">
       <c r="C19" s="3" t="s">
-        <v>123</v>
+        <v>79</v>
       </c>
       <c r="D19" s="50">
         <f>'Cone of Uncertainty'!E8-'Cone of Uncertainty'!E4</f>
@@ -25777,7 +25682,7 @@
     </row>
     <row r="21" spans="3:4" ht="16">
       <c r="C21" s="21" t="s">
-        <v>124</v>
+        <v>80</v>
       </c>
       <c r="D21" s="19">
         <v>2</v>
@@ -26050,49 +25955,65 @@
       <c r="B3" s="3">
         <v>1</v>
       </c>
-      <c r="C3" s="3"/>
+      <c r="C3" s="3" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="4" spans="2:3">
       <c r="B4" s="3">
         <v>2</v>
       </c>
-      <c r="C4" s="3"/>
+      <c r="C4" s="3" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="5" spans="2:3">
       <c r="B5" s="3">
         <v>3</v>
       </c>
-      <c r="C5" s="3"/>
+      <c r="C5" s="3" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="6" spans="2:3">
       <c r="B6" s="3">
         <v>4</v>
       </c>
-      <c r="C6" s="3"/>
+      <c r="C6" s="3" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="7" spans="2:3">
       <c r="B7" s="3">
         <v>5</v>
       </c>
-      <c r="C7" s="3"/>
+      <c r="C7" s="3" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="8" spans="2:3">
       <c r="B8" s="3">
         <v>6</v>
       </c>
-      <c r="C8" s="3"/>
+      <c r="C8" s="3" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="9" spans="2:3">
       <c r="B9" s="3">
         <v>7</v>
       </c>
-      <c r="C9" s="3"/>
+      <c r="C9" s="3" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="10" spans="2:3">
       <c r="B10" s="3">
         <v>8</v>
       </c>
-      <c r="C10" s="3"/>
+      <c r="C10" s="3" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="11" spans="2:3">
       <c r="B11" s="3">
@@ -26133,265 +26054,206 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:20" ht="19.25" customHeight="1">
-      <c r="A1" s="146" t="s">
-        <v>54</v>
-      </c>
-      <c r="B1" s="146"/>
-      <c r="C1" s="146"/>
-      <c r="D1" s="146"/>
-      <c r="E1" s="146"/>
-      <c r="F1" s="146"/>
-      <c r="G1" s="146"/>
-      <c r="H1" s="146"/>
-      <c r="I1" s="146"/>
-      <c r="J1" s="146"/>
-      <c r="K1" s="146"/>
-      <c r="L1" s="146"/>
-      <c r="M1" s="146"/>
-      <c r="N1" s="146"/>
-      <c r="O1" s="146"/>
-      <c r="P1" s="146"/>
-      <c r="Q1" s="146"/>
-      <c r="R1" s="146"/>
-      <c r="S1" s="146"/>
-      <c r="T1" s="146"/>
+      <c r="A1" s="149" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" s="149"/>
+      <c r="C1" s="149"/>
+      <c r="D1" s="149"/>
+      <c r="E1" s="149"/>
+      <c r="F1" s="149"/>
+      <c r="G1" s="149"/>
+      <c r="H1" s="149"/>
+      <c r="I1" s="149"/>
+      <c r="J1" s="149"/>
+      <c r="K1" s="149"/>
+      <c r="L1" s="149"/>
+      <c r="M1" s="149"/>
+      <c r="N1" s="149"/>
+      <c r="O1" s="149"/>
+      <c r="P1" s="149"/>
+      <c r="Q1" s="149"/>
+      <c r="R1" s="149"/>
+      <c r="S1" s="149"/>
+      <c r="T1" s="149"/>
     </row>
     <row r="2" spans="1:20" ht="29" customHeight="1">
-      <c r="A2" s="146"/>
-      <c r="B2" s="146"/>
-      <c r="C2" s="146"/>
-      <c r="D2" s="146"/>
-      <c r="E2" s="146"/>
-      <c r="F2" s="146"/>
-      <c r="G2" s="146"/>
-      <c r="H2" s="146"/>
-      <c r="I2" s="146"/>
-      <c r="J2" s="146"/>
-      <c r="K2" s="146"/>
-      <c r="L2" s="146"/>
-      <c r="M2" s="146"/>
-      <c r="N2" s="146"/>
-      <c r="O2" s="146"/>
-      <c r="P2" s="146"/>
-      <c r="Q2" s="146"/>
-      <c r="R2" s="146"/>
-      <c r="S2" s="146"/>
-      <c r="T2" s="146"/>
+      <c r="A2" s="149"/>
+      <c r="B2" s="149"/>
+      <c r="C2" s="149"/>
+      <c r="D2" s="149"/>
+      <c r="E2" s="149"/>
+      <c r="F2" s="149"/>
+      <c r="G2" s="149"/>
+      <c r="H2" s="149"/>
+      <c r="I2" s="149"/>
+      <c r="J2" s="149"/>
+      <c r="K2" s="149"/>
+      <c r="L2" s="149"/>
+      <c r="M2" s="149"/>
+      <c r="N2" s="149"/>
+      <c r="O2" s="149"/>
+      <c r="P2" s="149"/>
+      <c r="Q2" s="149"/>
+      <c r="R2" s="149"/>
+      <c r="S2" s="149"/>
+      <c r="T2" s="149"/>
     </row>
     <row r="4" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="A4" s="56" t="s">
-        <v>55</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B5" s="58" t="s">
-        <v>56</v>
+        <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B6" s="58" t="s">
-        <v>57</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B7" s="58" t="s">
-        <v>58</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:20" s="57" customFormat="1" ht="18">
-      <c r="B8" s="58" t="s">
-        <v>59</v>
-      </c>
+      <c r="A8" s="152" t="s">
+        <v>125</v>
+      </c>
+      <c r="B8" s="58"/>
     </row>
     <row r="9" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B9" s="58" t="s">
-        <v>60</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B10" s="58" t="s">
-        <v>61</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:20" s="57" customFormat="1" ht="18">
-      <c r="B11" s="58" t="s">
-        <v>62</v>
-      </c>
+      <c r="A11" s="152" t="s">
+        <v>128</v>
+      </c>
+      <c r="B11" s="58"/>
     </row>
     <row r="12" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B12" s="58" t="s">
-        <v>63</v>
+        <v>129</v>
       </c>
     </row>
     <row r="13" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B13" s="58" t="s">
-        <v>64</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:20" s="57" customFormat="1" ht="18">
-      <c r="B14" s="58" t="s">
-        <v>65</v>
-      </c>
+      <c r="A14" s="152" t="s">
+        <v>131</v>
+      </c>
+      <c r="B14" s="58"/>
     </row>
     <row r="15" spans="1:20" s="57" customFormat="1" ht="18">
       <c r="B15" s="58" t="s">
-        <v>66</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" spans="1:20" s="57" customFormat="1" ht="18">
-      <c r="A16" s="56" t="s">
-        <v>67</v>
-      </c>
+      <c r="A16" s="56"/>
     </row>
     <row r="17" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B17" s="58" t="s">
-        <v>68</v>
-      </c>
+      <c r="B17" s="58"/>
     </row>
     <row r="18" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B18" s="58" t="s">
-        <v>69</v>
-      </c>
+      <c r="B18" s="58"/>
     </row>
     <row r="19" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="A19" s="56" t="s">
-        <v>70</v>
-      </c>
+      <c r="A19" s="56"/>
     </row>
     <row r="20" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B20" s="58" t="s">
-        <v>71</v>
-      </c>
+      <c r="B20" s="58"/>
     </row>
     <row r="21" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B21" s="58" t="s">
-        <v>72</v>
-      </c>
+      <c r="B21" s="58"/>
     </row>
     <row r="22" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B22" s="58" t="s">
-        <v>73</v>
-      </c>
+      <c r="B22" s="58"/>
     </row>
     <row r="23" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B23" s="58" t="s">
-        <v>74</v>
-      </c>
+      <c r="B23" s="58"/>
     </row>
     <row r="24" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B24" s="58" t="s">
-        <v>75</v>
-      </c>
+      <c r="B24" s="58"/>
     </row>
     <row r="25" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B25" s="58" t="s">
-        <v>76</v>
-      </c>
+      <c r="B25" s="58"/>
     </row>
     <row r="26" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B26" s="58" t="s">
-        <v>77</v>
-      </c>
+      <c r="B26" s="58"/>
     </row>
     <row r="27" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B27" s="58" t="s">
-        <v>78</v>
-      </c>
+      <c r="B27" s="58"/>
     </row>
     <row r="28" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B28" s="58" t="s">
-        <v>79</v>
-      </c>
+      <c r="B28" s="58"/>
     </row>
     <row r="29" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B29" s="58" t="s">
-        <v>80</v>
-      </c>
+      <c r="B29" s="58"/>
     </row>
     <row r="30" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B30" s="58" t="s">
-        <v>81</v>
-      </c>
+      <c r="B30" s="58"/>
     </row>
     <row r="31" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B31" s="58" t="s">
-        <v>82</v>
-      </c>
+      <c r="B31" s="58"/>
     </row>
     <row r="32" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B32" s="58" t="s">
-        <v>83</v>
-      </c>
+      <c r="B32" s="58"/>
     </row>
     <row r="33" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B33" s="58" t="s">
-        <v>84</v>
-      </c>
+      <c r="B33" s="58"/>
     </row>
     <row r="34" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="A34" s="56" t="s">
-        <v>85</v>
-      </c>
+      <c r="A34" s="56"/>
     </row>
     <row r="35" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B35" s="58" t="s">
-        <v>86</v>
-      </c>
+      <c r="B35" s="58"/>
     </row>
     <row r="36" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B36" s="58" t="s">
-        <v>87</v>
-      </c>
+      <c r="B36" s="58"/>
     </row>
     <row r="37" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B37" s="58" t="s">
-        <v>88</v>
-      </c>
+      <c r="B37" s="58"/>
     </row>
     <row r="38" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="A38" s="56" t="s">
-        <v>89</v>
-      </c>
+      <c r="A38" s="56"/>
     </row>
     <row r="39" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B39" s="58" t="s">
-        <v>90</v>
-      </c>
+      <c r="B39" s="58"/>
     </row>
     <row r="40" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B40" s="58" t="s">
-        <v>91</v>
-      </c>
+      <c r="B40" s="58"/>
     </row>
     <row r="41" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B41" s="58" t="s">
-        <v>92</v>
-      </c>
+      <c r="B41" s="58"/>
     </row>
     <row r="42" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B42" s="58" t="s">
-        <v>93</v>
-      </c>
+      <c r="B42" s="58"/>
     </row>
     <row r="43" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B43" s="58" t="s">
-        <v>94</v>
-      </c>
+      <c r="B43" s="58"/>
     </row>
     <row r="44" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B44" s="58" t="s">
-        <v>95</v>
-      </c>
+      <c r="B44" s="58"/>
     </row>
     <row r="45" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B45" s="58" t="s">
-        <v>96</v>
-      </c>
+      <c r="B45" s="58"/>
     </row>
     <row r="46" spans="1:2" s="57" customFormat="1" ht="18">
-      <c r="B46" s="58" t="s">
-        <v>97</v>
-      </c>
+      <c r="B46" s="58"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -26424,101 +26286,101 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4">
-      <c r="B2" s="147" t="s">
-        <v>98</v>
-      </c>
-      <c r="C2" s="148"/>
-      <c r="D2" s="149"/>
+      <c r="B2" s="134" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="135"/>
+      <c r="D2" s="136"/>
     </row>
     <row r="3" spans="2:4" ht="14.25" customHeight="1">
       <c r="B3" s="116" t="s">
-        <v>99</v>
+        <v>55</v>
       </c>
       <c r="C3" s="116" t="s">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="D3" s="116" t="s">
-        <v>101</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="2:4">
       <c r="B4" s="3" t="s">
-        <v>128</v>
+        <v>84</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="D4" s="3"/>
     </row>
     <row r="5" spans="2:4">
       <c r="B5" s="3" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>103</v>
+        <v>59</v>
       </c>
       <c r="D5" s="3"/>
     </row>
     <row r="6" spans="2:4">
       <c r="B6" s="3" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>104</v>
+        <v>60</v>
       </c>
       <c r="D6" s="3"/>
     </row>
     <row r="7" spans="2:4">
       <c r="B7" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>104</v>
+        <v>60</v>
       </c>
       <c r="D7" s="3"/>
     </row>
     <row r="8" spans="2:4">
       <c r="B8" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>105</v>
+        <v>61</v>
       </c>
       <c r="D8" s="3"/>
     </row>
     <row r="9" spans="2:4">
       <c r="B9" s="3" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="D9" s="3"/>
     </row>
     <row r="10" spans="2:4">
       <c r="B10" s="3" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C10" s="27" t="s">
-        <v>107</v>
+        <v>63</v>
       </c>
       <c r="D10" s="27"/>
     </row>
     <row r="11" spans="2:4">
       <c r="B11" s="3" t="s">
-        <v>129</v>
+        <v>85</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>108</v>
+        <v>64</v>
       </c>
       <c r="D11" s="27"/>
     </row>
     <row r="12" spans="2:4">
       <c r="B12" s="3" t="s">
-        <v>130</v>
+        <v>86</v>
       </c>
       <c r="C12" s="27" t="s">
-        <v>109</v>
+        <v>65</v>
       </c>
       <c r="D12" s="27"/>
     </row>
@@ -26593,39 +26455,39 @@
     <row r="3" spans="2:20" ht="46.5" customHeight="1">
       <c r="B3" s="2"/>
       <c r="C3" s="116" t="s">
-        <v>110</v>
+        <v>66</v>
       </c>
       <c r="D3" s="115" t="s">
-        <v>111</v>
+        <v>67</v>
       </c>
       <c r="E3" s="115" t="s">
-        <v>112</v>
+        <v>68</v>
       </c>
       <c r="F3" s="115" t="s">
-        <v>113</v>
+        <v>69</v>
       </c>
       <c r="G3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="151" t="s">
-        <v>114</v>
+        <v>70</v>
       </c>
       <c r="K3" s="151"/>
       <c r="L3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="115" t="s">
-        <v>115</v>
+        <v>71</v>
       </c>
       <c r="P3" s="2"/>
       <c r="R3" s="2"/>
       <c r="S3" s="116" t="s">
-        <v>117</v>
+        <v>73</v>
       </c>
       <c r="T3" s="2"/>
     </row>
     <row r="4" spans="2:20">
       <c r="B4" s="2"/>
       <c r="C4" s="3" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="D4" s="11">
         <v>0</v>
@@ -26639,7 +26501,7 @@
       <c r="G4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="3" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="K4" s="1">
         <v>0</v>
@@ -26858,34 +26720,34 @@
     <row r="12" spans="2:20" ht="44.25" customHeight="1">
       <c r="B12" s="2"/>
       <c r="C12" s="116" t="s">
-        <v>110</v>
+        <v>66</v>
       </c>
       <c r="D12" s="115" t="s">
-        <v>119</v>
+        <v>75</v>
       </c>
       <c r="E12" s="115" t="s">
-        <v>120</v>
+        <v>76</v>
       </c>
       <c r="F12" s="115" t="s">
-        <v>121</v>
+        <v>77</v>
       </c>
       <c r="G12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="151" t="s">
-        <v>114</v>
+        <v>70</v>
       </c>
       <c r="K12" s="151"/>
       <c r="L12" s="2"/>
       <c r="N12" s="2"/>
       <c r="O12" s="115" t="s">
-        <v>116</v>
+        <v>72</v>
       </c>
       <c r="P12" s="2"/>
     </row>
     <row r="13" spans="2:20">
       <c r="B13" s="2"/>
       <c r="C13" s="3" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="D13" s="11">
         <v>0</v>
@@ -26902,7 +26764,7 @@
         <v>0</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>118</v>
+        <v>74</v>
       </c>
       <c r="L13" s="2"/>
       <c r="N13" s="2"/>
@@ -27147,21 +27009,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006DEE37CDC9AEA44CBD8F091652A6C5E4" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="9de09e14d18b2e0769f00e11c33b035a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7bb3299b-b075-41c7-bb54-99fc85b15d4f" xmlns:ns3="08caf6cd-a550-4dce-b6c8-fe9b0e6bc4e3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="81a6a9a579b993e4978c34f4e71e25a5" ns2:_="" ns3:_="">
     <xsd:import namespace="7bb3299b-b075-41c7-bb54-99fc85b15d4f"/>
@@ -27372,15 +27225,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1010AAFC-6E8A-4F4B-91D1-B1DB8DD7131E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF49F70C-261C-4E13-A8B5-F2B201AA0A03}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -27389,7 +27243,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D916E78-7E6F-4E04-B4AA-CEC365547DDB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -27406,4 +27260,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1010AAFC-6E8A-4F4B-91D1-B1DB8DD7131E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>